<commit_message>
[feat] attack pipline 代码修改
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
+++ b/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23540" windowHeight="14150"/>
+    <workbookView windowWidth="27945" windowHeight="11775"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>##var</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>order</t>
+  </si>
+  <si>
+    <t>maxStack</t>
   </si>
   <si>
     <t>##type</t>
@@ -996,15 +999,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5" outlineLevelCol="3"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="4"/>
   <cols>
-    <col min="2" max="2" width="17.3636363636364" style="1"/>
-    <col min="3" max="4" width="16.2727272727273" style="2"/>
-    <col min="5" max="5" width="30.4545454545455" customWidth="1"/>
+    <col min="2" max="2" width="17.3666666666667" style="1"/>
+    <col min="3" max="4" width="16.275" style="2"/>
+    <col min="5" max="5" width="30.4583333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1017,51 +1020,63 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="B5" s="1">
         <v>1002000001</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
       </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="B6" s="1">
         <v>1002000002</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2">
         <v>2</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1075,7 +1090,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1087,7 +1102,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
[wip] buff pipline 4
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
+++ b/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11775"/>
+    <workbookView windowWidth="25420" windowHeight="13410"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
   <si>
     <t>##var</t>
   </si>
@@ -40,10 +40,10 @@
     <t>##别称</t>
   </si>
   <si>
-    <t>order</t>
-  </si>
-  <si>
-    <t>maxStack</t>
+    <t>effects</t>
+  </si>
+  <si>
+    <t>parametric</t>
   </si>
   <si>
     <t>##type</t>
@@ -52,13 +52,31 @@
     <t>int</t>
   </si>
   <si>
+    <t>array#sep=|,string</t>
+  </si>
+  <si>
+    <t>map,Battle.BuffParam,float</t>
+  </si>
+  <si>
     <t>##</t>
   </si>
   <si>
     <t>唯一id</t>
   </si>
   <si>
+    <t>Buff参数</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
     <t>冻伤</t>
+  </si>
+  <si>
+    <t>初始层数</t>
+  </si>
+  <si>
+    <t>计时</t>
   </si>
   <si>
     <t>流血</t>
@@ -678,7 +696,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -687,6 +705,9 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -999,15 +1020,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="4"/>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
-    <col min="2" max="2" width="17.3666666666667" style="1"/>
-    <col min="3" max="4" width="16.275" style="2"/>
-    <col min="5" max="5" width="30.4583333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.3636363636364" style="1"/>
+    <col min="3" max="3" width="16.2727272727273" style="2"/>
+    <col min="4" max="4" width="20.8181818181818" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.18181818181818" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1020,11 +1042,18 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1032,54 +1061,101 @@
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:12">
       <c r="B5" s="1">
         <v>1002000001</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:12">
       <c r="B6" s="1">
         <v>1002000002</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2</v>
-      </c>
-      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E1:L1"/>
+    <mergeCell ref="E2:L2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
@@ -1090,7 +1166,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1102,7 +1178,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>